<commit_message>
Planilla por país: los 20 países ILIA + marcar SIN CASOS (JM, SV)
La planilla por país ahora incluye pestaña para los 20 países del ILIA (no solo
los que tienen casos). Jamaica (JM) y El Salvador (SV) no tienen casos este ciclo:
se marcan «SIN CASOS» en el índice de Instrucciones y con una pestaña-nota para
que el partner confirme o agregue. 22 pestañas (20 países + LATAM + Instrucciones).

Verificación de URLs en curso (5 agentes) para la planilla de partners.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMPcjwdKJwtrGXbXxDZgrC
</commit_message>
<xml_diff>
--- a/data/gates/planilla_validacion_por_pais_ILIA2026.xlsx
+++ b/data/gates/planilla_validacion_por_pais_ILIA2026.xlsx
@@ -19,14 +19,16 @@
     <sheet name="EC - Ecuador" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="GT - Guatemala" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="HN - Honduras" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="MX - México" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="PA - Panamá" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="PE - Perú" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="PY - Paraguay" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="TT - Trinidad y Tobago" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="UY - Uruguay" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="VE - Venezuela" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="LATAM - Regional" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="JM - Jamaica" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="MX - México" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="PA - Panamá" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="PE - Perú" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="PY - Paraguay" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="SV - El Salvador" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="TT - Trinidad y Tobago" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="UY - Uruguay" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="VE - Venezuela" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="LATAM - Regional" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'AR - Argentina'!$A$1:$F$6</definedName>
@@ -40,14 +42,16 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'EC - Ecuador'!$A$1:$F$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'GT - Guatemala'!$A$1:$F$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'HN - Honduras'!$A$1:$F$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'MX - México'!$A$1:$F$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'PA - Panamá'!$A$1:$F$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'PE - Perú'!$A$1:$F$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'PY - Paraguay'!$A$1:$F$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'TT - Trinidad y Tobago'!$A$1:$F$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'UY - Uruguay'!$A$1:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'VE - Venezuela'!$A$1:$F$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'LATAM - Regional'!$A$1:$F$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'JM - Jamaica'!$A$1:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'MX - México'!$A$1:$F$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'PA - Panamá'!$A$1:$F$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'PE - Perú'!$A$1:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'PY - Paraguay'!$A$1:$F$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'SV - El Salvador'!$A$1:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'TT - Trinidad y Tobago'!$A$1:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'UY - Uruguay'!$A$1:$F$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'VE - Venezuela'!$A$1:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'LATAM - Regional'!$A$1:$F$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -521,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -607,139 +611,131 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>ÍNDICE</t>
+          <t>Cobertura</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>País — casos (de los cuales SÍ / DUDA / NO)</t>
+          <t>Los 20 países del ILIA tienen pestaña. Los que no tienen casos identificados este ciclo se marcan «SIN CASOS» (por favor confirme si conoce alguno).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>AR — Argentina</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>5 casos  (SÍ 0 · DUDA 0 · NO 5)</t>
-        </is>
-      </c>
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>BO — Bolivia</t>
+          <t>ÍNDICE (20 países ILIA + Regional)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>1 casos  (SÍ 1 · DUDA 0 · NO 0)</t>
+          <t>País — casos (de los cuales SÍ / DUDA / NO)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>BR — Brasil</t>
+          <t>AR — Argentina</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>23 casos  (SÍ 9 · DUDA 0 · NO 14)</t>
+          <t>5 casos  (SÍ 0 · DUDA 0 · NO 5)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>CL — Chile</t>
+          <t>BO — Bolivia</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>17 casos  (SÍ 10 · DUDA 2 · NO 5)</t>
+          <t>1 casos  (SÍ 1 · DUDA 0 · NO 0)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>CO — Colombia</t>
+          <t>BR — Brasil</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>19 casos  (SÍ 4 · DUDA 1 · NO 14)</t>
+          <t>23 casos  (SÍ 9 · DUDA 0 · NO 14)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>CR — Costa Rica</t>
+          <t>CL — Chile</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2 casos  (SÍ 0 · DUDA 0 · NO 2)</t>
+          <t>17 casos  (SÍ 10 · DUDA 2 · NO 5)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>CU — Cuba</t>
+          <t>CO — Colombia</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>1 casos  (SÍ 0 · DUDA 0 · NO 1)</t>
+          <t>19 casos  (SÍ 4 · DUDA 1 · NO 14)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>DO — Rep. Dominicana</t>
+          <t>CR — Costa Rica</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>3 casos  (SÍ 0 · DUDA 0 · NO 3)</t>
+          <t>2 casos  (SÍ 0 · DUDA 0 · NO 2)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>EC — Ecuador</t>
+          <t>CU — Cuba</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>1 casos  (SÍ 1 · DUDA 0 · NO 0)</t>
+          <t>1 casos  (SÍ 0 · DUDA 0 · NO 1)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>GT — Guatemala</t>
+          <t>DO — Rep. Dominicana</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>2 casos  (SÍ 1 · DUDA 0 · NO 1)</t>
+          <t>3 casos  (SÍ 0 · DUDA 0 · NO 3)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>HN — Honduras</t>
+          <t>EC — Ecuador</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -751,96 +747,160 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>MX — México</t>
+          <t>GT — Guatemala</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>14 casos  (SÍ 2 · DUDA 1 · NO 11)</t>
+          <t>2 casos  (SÍ 1 · DUDA 0 · NO 1)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>PA — Panamá</t>
+          <t>HN — Honduras</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2 casos  (SÍ 1 · DUDA 0 · NO 1)</t>
+          <t>1 casos  (SÍ 1 · DUDA 0 · NO 0)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>PE — Perú</t>
+          <t>JM — Jamaica</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>3 casos  (SÍ 1 · DUDA 0 · NO 2)</t>
+          <t>SIN CASOS identificados este ciclo</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>PY — Paraguay</t>
+          <t>MX — México</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>2 casos  (SÍ 0 · DUDA 0 · NO 2)</t>
+          <t>14 casos  (SÍ 2 · DUDA 1 · NO 11)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>TT — Trinidad y Tobago</t>
+          <t>PA — Panamá</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>1 casos  (SÍ 1 · DUDA 0 · NO 0)</t>
+          <t>2 casos  (SÍ 1 · DUDA 0 · NO 1)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>UY — Uruguay</t>
+          <t>PE — Perú</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>4 casos  (SÍ 1 · DUDA 0 · NO 3)</t>
+          <t>3 casos  (SÍ 1 · DUDA 0 · NO 2)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>VE — Venezuela</t>
+          <t>PY — Paraguay</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>1 casos  (SÍ 0 · DUDA 0 · NO 1)</t>
+          <t>2 casos  (SÍ 0 · DUDA 0 · NO 2)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
+          <t>SV — El Salvador</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>SIN CASOS identificados este ciclo</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>TT — Trinidad y Tobago</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>1 casos  (SÍ 1 · DUDA 0 · NO 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>UY — Uruguay</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>4 casos  (SÍ 1 · DUDA 0 · NO 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>VE — Venezuela</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>1 casos  (SÍ 0 · DUDA 0 · NO 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
           <t>LATAM — LATAM / Regional</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>5 casos  (SÍ 0 · DUDA 0 · NO 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr"/>
+      <c r="B33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Países SIN casos</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>JM (Jamaica), SV (El Salvador)</t>
         </is>
       </c>
     </row>
@@ -1120,6 +1180,81 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Caso</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Descripción breve</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Fuente (URL validada)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>¿Se incluye?</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Motivo (si NO/DUDA)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Comentario / corrección (partner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>(sin casos identificados este ciclo)</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>No se identificaron casos de IA en participación ciudadana para este país. Si conoce alguno, agréguelo en las filas de abajo.</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr"/>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr"/>
+      <c r="F2" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1553,7 +1688,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1660,7 +1795,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1795,7 +1930,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1906,7 +2041,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1958,22 +2093,18 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>EngageTT (engage.gov.tt) sobre plataforma Go Vocal (antes CitizenLab) - consulta del National Digital Transformation Strategy (NDTS) 2024-2027</t>
+          <t>(sin casos identificados este ciclo)</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>EngageTT (engage.gov.tt) es la plataforma de participacion ciudadana del Ministry of Digital Transformation de Trinidad y Tobago (desde mayo 2025 fusionado en el Ministry of Public Administration and Artificial Intelligence, MP…</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>https://support.govocal.com/en/articles/8316692-ai-analysis</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>SÍ</t>
+          <t>No se identificaron casos de IA en participación ciudadana para este país. Si conoce alguno, agréguelo en las filas de abajo.</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr"/>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr"/>
@@ -1981,169 +2112,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:F2"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Caso</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Descripción breve</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Fuente (URL validada)</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>¿Se incluye?</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Motivo (si NO/DUDA)</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Comentario / corrección (partner)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Pol.is en el Referéndum Nacional de la LUC (Uruguay) — equipo UdelaR</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>Referéndum nacional para derogar 135 artículos de la Ley de Urgente Consideración (LUC).</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>https://compdemocracy.org/case-studies/2021-uruguay-national-referendum/</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr"/>
-      <c r="F2" s="5" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Chatbot (Asistente virtual entrenado con IA)</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Asistente Virtual de AGESIC – Chatbot gubernamental piloto lanzado en 2018 para adquirir experiencia en soluciones de IA en la atención ciudadana.</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>https://www.oecd.org/content/dam/oecd/es/publications/reports/2022/03/the-strategic-and-responsible-use-of-artificial-intelligence-in-the-public-sector-of-latin-america-and-the-caribbean_17c90e5e/5b189cb4-es.pdf#:~:text=El%20chatbot%20virtual%20creado%20por,desarrollo%20de%20soluciones%20de%20IA</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Atencion ciudadana</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Consulta Pública de la Estrategia Nacional de Inteligencia Artificial (IA) de Uruguay 2024–2030,</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Es una iniciativa del gobierno uruguayo para definir una política pública de IA que abarque los sectores público, privado, académico y de la sociedad civil.</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>https://www.gub.uy/agencia-gobierno-electronico-sociedad-informacion-conocimiento/comunicacion/publicaciones/estrategia-nacional-inteligencia-artificial-2024-2030?utm_source=chatgpt.com</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>No evidencia de uso de IA</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Consulta Pública y Participación Multiactores: "Niñas, niños, adolescentes, entornos digitales e inteligencia artificial" (Uruguay, 2026)</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Consulta pública nacional y participación multiactores impulsada por el Parlamento de Uruguay junto a Agesic, el Consejo Nacional Consultivo Honorario de los Derechos de la Niñez y la Adolescencia, Ceibal, UNICEF y PNUD.</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>https://www.gub.uy/ministerio-educacion-cultura/comunicacion/noticias/lanzamiento-consulta-publica-sobre-inteligencia-artificial-entornos-digitales</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>NO (lean firme). (1) TEMPORAL: la consulta está ABIERTA hasta el 10/09/2026 y la fase de sistematización/análisis/validación (Fase 3) recién ocurre entre el 10/09 y el 10/10/2026, con informe final el</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2200,29 +2168,25 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Plan de la Patria 7 Transformaciones (7T) - IA y Big Data en la sistematización de propuestas de la Consulta Popular</t>
+          <t>EngageTT (engage.gov.tt) sobre plataforma Go Vocal (antes CitizenLab) - consulta del National Digital Transformation Strategy (NDTS) 2024-2027</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Proceso de consulta/debate para la elaboración del Plan de la Patria de las 7 Grandes Transformaciones (7T) 2025-2031, conducido por el Gobierno Bolivariano de Venezuela (Ministerio del Poder Popular de Planificación / Vicepres…</t>
+          <t>EngageTT (engage.gov.tt) es la plataforma de participacion ciudadana del Ministry of Digital Transformation de Trinidad y Tobago (desde mayo 2025 fusionado en el Ministry of Public Administration and Artificial Intelligence, MP…</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>http://www.correodelorinoco.gob.ve/venezuela-impulsa-el-debate-sobre-inteligencia-artificial-bajo-principios-de-soberania-y-etica/</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>NO (resuelto en 2ª pasada, antes DUDA). Hay un proceso participativo claro (consulta/debate nacional para construir el Plan de la Patria 7T, con +63.000 asambleas, 3,4 M de participantes y 34.491 prop</t>
-        </is>
-      </c>
+          <t>https://support.govocal.com/en/articles/8316692-ai-analysis</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr"/>
       <c r="F2" s="5" t="inlineStr"/>
     </row>
   </sheetData>
@@ -2432,6 +2396,252 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Caso</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Descripción breve</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Fuente (URL validada)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>¿Se incluye?</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Motivo (si NO/DUDA)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Comentario / corrección (partner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Pol.is en el Referéndum Nacional de la LUC (Uruguay) — equipo UdelaR</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Referéndum nacional para derogar 135 artículos de la Ley de Urgente Consideración (LUC).</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>https://compdemocracy.org/case-studies/2021-uruguay-national-referendum/</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr"/>
+      <c r="F2" s="5" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Chatbot (Asistente virtual entrenado con IA)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Asistente Virtual de AGESIC – Chatbot gubernamental piloto lanzado en 2018 para adquirir experiencia en soluciones de IA en la atención ciudadana.</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>https://www.oecd.org/content/dam/oecd/es/publications/reports/2022/03/the-strategic-and-responsible-use-of-artificial-intelligence-in-the-public-sector-of-latin-america-and-the-caribbean_17c90e5e/5b189cb4-es.pdf#:~:text=El%20chatbot%20virtual%20creado%20por,desarrollo%20de%20soluciones%20de%20IA</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Atencion ciudadana</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Consulta Pública de la Estrategia Nacional de Inteligencia Artificial (IA) de Uruguay 2024–2030,</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Es una iniciativa del gobierno uruguayo para definir una política pública de IA que abarque los sectores público, privado, académico y de la sociedad civil.</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gub.uy/agencia-gobierno-electronico-sociedad-informacion-conocimiento/comunicacion/publicaciones/estrategia-nacional-inteligencia-artificial-2024-2030?utm_source=chatgpt.com</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>No evidencia de uso de IA</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Consulta Pública y Participación Multiactores: "Niñas, niños, adolescentes, entornos digitales e inteligencia artificial" (Uruguay, 2026)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Consulta pública nacional y participación multiactores impulsada por el Parlamento de Uruguay junto a Agesic, el Consejo Nacional Consultivo Honorario de los Derechos de la Niñez y la Adolescencia, Ceibal, UNICEF y PNUD.</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>https://www.gub.uy/ministerio-educacion-cultura/comunicacion/noticias/lanzamiento-consulta-publica-sobre-inteligencia-artificial-entornos-digitales</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>NO (lean firme). (1) TEMPORAL: la consulta está ABIERTA hasta el 10/09/2026 y la fase de sistematización/análisis/validación (Fase 3) recién ocurre entre el 10/09 y el 10/10/2026, con informe final el</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F5"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Caso</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Descripción breve</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Fuente (URL validada)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>¿Se incluye?</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Motivo (si NO/DUDA)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Comentario / corrección (partner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Plan de la Patria 7 Transformaciones (7T) - IA y Big Data en la sistematización de propuestas de la Consulta Popular</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Proceso de consulta/debate para la elaboración del Plan de la Patria de las 7 Grandes Transformaciones (7T) 2025-2031, conducido por el Gobierno Bolivariano de Venezuela (Ministerio del Poder Popular de Planificación / Vicepres…</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>http://www.correodelorinoco.gob.ve/venezuela-impulsa-el-debate-sobre-inteligencia-artificial-bajo-principios-de-soberania-y-etica/</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>NO (resuelto en 2ª pasada, antes DUDA). Hay un proceso participativo claro (consulta/debate nacional para construir el Plan de la Patria 7T, con +63.000 asambleas, 3,4 M de participantes y 34.491 prop</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Verificar y corregir todas las URLs de la planilla por país (partners)
Verificación de las 107 URLs con 5 agentes (vía WebSearch-indexación, ya que
curl/WebFetch salen bloqueados por la política de egress del entorno). Resultado:
107/107 reales e indexadas; 0 rotas / 0 inventadas tras las correcciones.

Rotas corregidas (7): CL Estudio dIAlogos (slug ES→/en/+estudiodialogos.cl),
CL Jornada UNAB (Tableau→ipp.unab.cl), DO Sara (slug -0 roto→undp guatemala),
EC PAGA IA (boletin-014 inexistente→ia.gobiernoabierto.ec), PE Consulta
(LATINNO 17232→gob.pe/cne), LATAM ANTAI/CAF (+/2021/07/), LATAM Chatbot DCI (+-1).
Robustecidas (5): informe OCDE PDF→URL canónica; clustering→arXiv 2509.21292;
Viña Decide→vinadecide.cl; ParaEmpleo→/en/; Sufragio seguro→algoritmoscide.org.
+8 URLs con tracking utm limpiadas.

Nuevo doc verificacion_urls_por_pais_ILIA2026.md.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMPcjwdKJwtrGXbXxDZgrC
</commit_message>
<xml_diff>
--- a/data/gates/planilla_validacion_por_pais_ILIA2026.xlsx
+++ b/data/gates/planilla_validacion_por_pais_ILIA2026.xlsx
@@ -971,7 +971,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>https://www.gobiernoabierto.ec/boletin-014-2023/</t>
+          <t>https://ia.gobiernoabierto.ec/</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/content/dam/oecd/es/publications/reports/2022/03/the-strategic-and-responsible-use-of-artificial-intelligence-in-the-public-sector-of-latin-america-and-the-caribbean_17c90e5e/5b189cb4-es.pdf#:~:text=para%20identificar%20posibles%20trastornos,de%20las%20dificultades%20de%20%C3%ADndole</t>
+          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>https://osf.io/cu6w3</t>
+          <t>https://algoritmoscide.org/proyectos/sufragio-seguro/</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/content/dam/oecd/es/publications/reports/2022/03/the-strategic-and-responsible-use-of-artificial-intelligence-in-the-public-sector-of-latin-america-and-the-caribbean_17c90e5e/5b189cb4-es.pdf#:~:text=virtual%2Fchatbot%20que%20funciona%20por%20WhatsApp,que%20realice%20una%20observaci%C3%B3n%20f%C3%ADsica</t>
+          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>https://www.latinno.net/en/case/17232/</t>
+          <t>https://www.gob.pe/institucion/cne/noticias/502734-lanzan-consulta-ciudadana-por-el-proyecto-educativo-nacional</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>https://fairlac.iadb.org/paraempleo</t>
+          <t>https://fairlac.iadb.org/en/paraempleo</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/content/dam/oecd/es/publications/reports/2022/03/the-strategic-and-responsible-use-of-artificial-intelligence-in-the-public-sector-of-latin-america-and-the-caribbean_17c90e5e/5b189cb4-es.pdf#:~:text=El%20chatbot%20virtual%20creado%20por,desarrollo%20de%20soluciones%20de%20IA</t>
+          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>https://www.gub.uy/agencia-gobierno-electronico-sociedad-informacion-conocimiento/comunicacion/publicaciones/estrategia-nacional-inteligencia-artificial-2024-2030?utm_source=chatgpt.com</t>
+          <t>https://www.gub.uy/agencia-gobierno-electronico-sociedad-informacion-conocimiento/comunicacion/publicaciones/estrategia-nacional-inteligencia-artificial-2024-2030</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -2698,7 +2698,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>https://www.caf.com/es/actualidad/noticias/caf-realiza-su-primera-inversion-en-una-govtech-latinoamericana/</t>
+          <t>https://www.caf.com/es/actualidad/noticias/2021/07/caf-realiza-su-primera-inversion-en-una-govtech-latinoamericana/</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>https://www.policylab.tech/post/revolucionando-la-denuncia-ciudadana-en-am%C3%A9rica-latina-con-tecnolog%C3%ADa-el-caso-del-chatbot-dci</t>
+          <t>https://www.policylab.tech/post/revolucionando-la-denuncia-ciudadana-en-am%C3%A9rica-latina-con-tecnolog%C3%ADa-el-caso-del-chatbot-dci-1</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -2996,7 +2996,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2511.01545</t>
+          <t>https://arxiv.org/abs/2509.21292</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
@@ -3304,7 +3304,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>https://www.oecd.org/content/dam/oecd/es/publications/reports/2022/03/the-strategic-and-responsible-use-of-artificial-intelligence-in-the-public-sector-of-latin-america-and-the-caribbean_17c90e5e/5b189cb4-es.pdf#:~:text=Jaque%20y%20la%20Gu%C3%ADa%20de,Contiene%20informaci%C3%B3n%2C%20entre</t>
+          <t>https://www.oecd.org/es/publications/uso-estrategico-y-responsable-de-la-inteligencia-artificial-en-el-sector-publico-de-america-latina-y-el-caribe_5b189cb4-es/full-report.html</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -3687,7 +3687,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>https://participacion.digital.gob.cl/es-CL/folders/consultas-ciudadanas</t>
+          <t>https://participacion.digital.gob.cl/projects/segunda-consulta-estrategia-de-gobierno-digital-2030</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>https://fairlac.iadb.org/estudio-dialogos-percepciones-de-futuro</t>
+          <t>https://estudiodialogos.cl/</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -3735,7 +3735,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>https://public.tableau.com/app/profile/ivania.yovanovic/viz/JornadasInstitutoPolticasPblicasUNAB/Dashboard3</t>
+          <t>https://ipp.unab.cl/</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -3907,7 +3907,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>https://arxiv.org/abs/2303.15532?utm_source=chatgpt.com</t>
+          <t>https://arxiv.org/abs/2303.15532</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -4047,7 +4047,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>https://www.govocal.com/</t>
+          <t>https://vinadecide.cl/pages/presupuestoparticipativo</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>https://projects.itforchange.net/mavc/wp-content/uploads/2017/09/Voice-or-Chatter_Case-Study_Colombia_August-2017.pdf?utm_source=chatgpt.com</t>
+          <t>https://projects.itforchange.net/mavc/wp-content/uploads/2017/09/Voice-or-Chatter_Case-Study_Colombia_August-2017.pdf</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -4923,7 +4923,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>https://www.undp.org/es/latin-america/comunicados-de-prensa/sara-la-nueva-herramienta-de-inteligencia-artificial-para-combatir-la-violencia-de-genero-en-centroamerica-0</t>
+          <t>https://www.undp.org/es/guatemala/comunicados-de-prensa/sara-la-nueva-herramienta-de-inteligencia-artificial-para-combatir-la-violencia-de-genero-en-centroamerica</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">

</xml_diff>